<commit_message>
Rename Alfa Romeo paint to Alfa Rosso
</commit_message>
<xml_diff>
--- a/data/source/Car_Paint_Colors_v4.xlsx
+++ b/data/source/Car_Paint_Colors_v4.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Colors" sheetId="1" r:id="R6eaf113865ef4843"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="2" r:id="R5ecc28ae532c4062"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema &amp; Notes" sheetId="3" r:id="Reb29f42bbb104c1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Colors" sheetId="1" r:id="R208dab38d926404e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="2" r:id="Re3e8544289d7478f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema &amp; Notes" sheetId="3" r:id="Rcd73a7098f11454c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23274,7 +23274,7 @@
       <x:c r="F265" s="1234"/>
       <x:c r="G265" s="1234"/>
       <x:c r="H265" s="1238" t="str">
-        <x:v>Alfa Red car paint</x:v>
+        <x:v>Alfa Rosso</x:v>
       </x:c>
       <x:c r="I265" s="1236" t="str">
         <x:v>414A</x:v>
@@ -23294,7 +23294,7 @@
       <x:c r="N265" s="1248"/>
       <x:c r="O265" s="1248"/>
       <x:c r="P265" s="1246" t="str">
-        <x:v>OEM code confirmed on paintref for Giulia/Stelvio; hex estimated</x:v>
+        <x:v>OEM code confirmed on paintref for Giulia/Stelvio; hex estimated; Original source label: Alfa Red car paint.</x:v>
       </x:c>
       <x:c r="Q265" s="1482" t="str">
         <x:v>Estimated</x:v>

</xml_diff>